<commit_message>
Change column names to match nee Rate importer columns
</commit_message>
<xml_diff>
--- a/landing_zone/2026/Honda/2025-06/2026-Honda_Master-06_2025.xlsx
+++ b/landing_zone/2026/Honda/2025-06/2026-Honda_Master-06_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pbssystems-my.sharepoint.com/personal/paxm_pbssystems_com/Documents/Desktop/Office/Projects/OEM Accessory project/OEM Accessories_v1/landing_zone/2026/2025-06/Honda/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pbssystems-my.sharepoint.com/personal/paxm_pbssystems_com/Documents/Desktop/Office/Projects/OEM Accessory project/OEM Accessories_v1/landing_zone/2026/Honda/2025-06/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{072DAD4C-14B6-4D03-B94B-C4050A756E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E09274D7-BC02-4968-B7A4-4EF36DC7DAB5}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{072DAD4C-14B6-4D03-B94B-C4050A756E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4B24E98-25B6-437E-9AF7-4CA6925FDCD0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRV Master" sheetId="15" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CRV Master'!$G$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HRV Master'!$E$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Passport Master'!$E$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Passport Master'!$E$1:$J$62</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2396" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2395" uniqueCount="745">
   <si>
     <t>Description</t>
   </si>
@@ -1982,9 +1982,6 @@
     <t>26PAS-RUGPK</t>
   </si>
   <si>
-    <t>$ 2,552.00</t>
-  </si>
-  <si>
     <t>1.9</t>
   </si>
   <si>
@@ -2400,8 +2397,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -2495,7 +2493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2520,6 +2518,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2535,10 +2534,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2898,7 +2893,7 @@
         <v>0</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="I1" s="9" t="s">
         <v>1</v>
@@ -6430,16 +6425,16 @@
   <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" customWidth="1"/>
     <col min="9" max="9" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="131.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="91.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="45" x14ac:dyDescent="0.25">
@@ -6459,7 +6454,7 @@
         <v>0</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -6653,17 +6648,17 @@
       <c r="F7" t="s">
         <v>609</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="12">
+        <v>2552</v>
+      </c>
+      <c r="H7" t="s">
+        <v>611</v>
+      </c>
+      <c r="I7" t="s">
         <v>610</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>612</v>
-      </c>
-      <c r="I7" t="s">
-        <v>611</v>
-      </c>
-      <c r="J7" t="s">
-        <v>613</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -6683,19 +6678,19 @@
         <v>17</v>
       </c>
       <c r="F8" t="s">
+        <v>613</v>
+      </c>
+      <c r="G8" t="s">
         <v>614</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>615</v>
-      </c>
-      <c r="H8" t="s">
-        <v>616</v>
       </c>
       <c r="I8" t="s">
         <v>46</v>
       </c>
       <c r="J8" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -6712,16 +6707,16 @@
         <v>525</v>
       </c>
       <c r="E9" t="s">
+        <v>617</v>
+      </c>
+      <c r="F9" t="s">
         <v>618</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>619</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>620</v>
-      </c>
-      <c r="H9" t="s">
-        <v>621</v>
       </c>
       <c r="I9" t="s">
         <v>241</v>
@@ -6747,13 +6742,13 @@
         <v>27</v>
       </c>
       <c r="F10" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="G10" t="s">
         <v>204</v>
       </c>
       <c r="H10" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="I10" t="s">
         <v>9</v>
@@ -6776,13 +6771,13 @@
         <v>23</v>
       </c>
       <c r="F11" t="s">
+        <v>623</v>
+      </c>
+      <c r="G11" t="s">
         <v>624</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>625</v>
-      </c>
-      <c r="H11" t="s">
-        <v>626</v>
       </c>
       <c r="I11" t="s">
         <v>9</v>
@@ -6802,16 +6797,16 @@
         <v>525</v>
       </c>
       <c r="E12" t="s">
+        <v>626</v>
+      </c>
+      <c r="F12" t="s">
         <v>627</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>628</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>629</v>
-      </c>
-      <c r="H12" t="s">
-        <v>630</v>
       </c>
       <c r="I12" t="s">
         <v>84</v>
@@ -6831,16 +6826,16 @@
         <v>525</v>
       </c>
       <c r="E13" t="s">
+        <v>630</v>
+      </c>
+      <c r="F13" t="s">
         <v>631</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>632</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>633</v>
-      </c>
-      <c r="H13" t="s">
-        <v>634</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -6860,22 +6855,22 @@
         <v>525</v>
       </c>
       <c r="E14" t="s">
+        <v>634</v>
+      </c>
+      <c r="F14" t="s">
         <v>635</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>636</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>637</v>
-      </c>
-      <c r="H14" t="s">
-        <v>638</v>
       </c>
       <c r="I14" t="s">
         <v>15</v>
       </c>
       <c r="J14" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -6895,19 +6890,19 @@
         <v>302</v>
       </c>
       <c r="F15" t="s">
+        <v>639</v>
+      </c>
+      <c r="G15" t="s">
         <v>640</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>641</v>
-      </c>
-      <c r="H15" t="s">
-        <v>642</v>
       </c>
       <c r="I15" t="s">
         <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -6924,16 +6919,16 @@
         <v>525</v>
       </c>
       <c r="E16" t="s">
+        <v>643</v>
+      </c>
+      <c r="F16" t="s">
         <v>644</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>645</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>646</v>
-      </c>
-      <c r="H16" t="s">
-        <v>647</v>
       </c>
       <c r="I16" t="s">
         <v>90</v>
@@ -6953,16 +6948,16 @@
         <v>525</v>
       </c>
       <c r="E17" t="s">
+        <v>647</v>
+      </c>
+      <c r="F17" t="s">
         <v>648</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>649</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>650</v>
-      </c>
-      <c r="H17" t="s">
-        <v>651</v>
       </c>
       <c r="I17" t="s">
         <v>72</v>
@@ -6982,16 +6977,16 @@
         <v>525</v>
       </c>
       <c r="E18" t="s">
+        <v>651</v>
+      </c>
+      <c r="F18" t="s">
         <v>652</v>
-      </c>
-      <c r="F18" t="s">
-        <v>653</v>
       </c>
       <c r="G18" t="s">
         <v>197</v>
       </c>
       <c r="H18" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="I18" t="s">
         <v>72</v>
@@ -7014,13 +7009,13 @@
         <v>331</v>
       </c>
       <c r="F19" t="s">
+        <v>654</v>
+      </c>
+      <c r="G19" t="s">
         <v>655</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>656</v>
-      </c>
-      <c r="H19" t="s">
-        <v>657</v>
       </c>
       <c r="I19" t="s">
         <v>72</v>
@@ -7043,13 +7038,13 @@
         <v>86</v>
       </c>
       <c r="F20" t="s">
+        <v>657</v>
+      </c>
+      <c r="G20" t="s">
         <v>658</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>659</v>
-      </c>
-      <c r="H20" t="s">
-        <v>660</v>
       </c>
       <c r="I20" t="s">
         <v>15</v>
@@ -7069,16 +7064,16 @@
         <v>529</v>
       </c>
       <c r="E21" t="s">
+        <v>660</v>
+      </c>
+      <c r="F21" t="s">
         <v>661</v>
-      </c>
-      <c r="F21" t="s">
-        <v>662</v>
       </c>
       <c r="G21" t="s">
         <v>200</v>
       </c>
       <c r="H21" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="I21" t="s">
         <v>84</v>
@@ -7098,16 +7093,16 @@
         <v>529</v>
       </c>
       <c r="E22" t="s">
+        <v>663</v>
+      </c>
+      <c r="F22" t="s">
         <v>664</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>665</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>666</v>
-      </c>
-      <c r="H22" t="s">
-        <v>667</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
@@ -7127,10 +7122,10 @@
         <v>525</v>
       </c>
       <c r="E23" t="s">
+        <v>667</v>
+      </c>
+      <c r="F23" t="s">
         <v>668</v>
-      </c>
-      <c r="F23" t="s">
-        <v>669</v>
       </c>
       <c r="G23" t="s">
         <v>204</v>
@@ -7156,16 +7151,16 @@
         <v>525</v>
       </c>
       <c r="E24" t="s">
+        <v>669</v>
+      </c>
+      <c r="F24" t="s">
         <v>670</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>671</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>672</v>
-      </c>
-      <c r="H24" t="s">
-        <v>673</v>
       </c>
       <c r="I24" t="s">
         <v>566</v>
@@ -7188,10 +7183,10 @@
         <v>355</v>
       </c>
       <c r="F25" t="s">
+        <v>673</v>
+      </c>
+      <c r="G25" t="s">
         <v>674</v>
-      </c>
-      <c r="G25" t="s">
-        <v>675</v>
       </c>
       <c r="H25" t="s">
         <v>357</v>
@@ -7217,10 +7212,10 @@
         <v>358</v>
       </c>
       <c r="F26" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="G26" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="H26" t="s">
         <v>357</v>
@@ -7249,7 +7244,7 @@
         <v>140</v>
       </c>
       <c r="G27" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H27" t="s">
         <v>141</v>
@@ -7275,13 +7270,13 @@
         <v>364</v>
       </c>
       <c r="F28" t="s">
+        <v>677</v>
+      </c>
+      <c r="G28" t="s">
+        <v>658</v>
+      </c>
+      <c r="H28" t="s">
         <v>678</v>
-      </c>
-      <c r="G28" t="s">
-        <v>659</v>
-      </c>
-      <c r="H28" t="s">
-        <v>679</v>
       </c>
       <c r="I28" t="s">
         <v>84</v>
@@ -7301,16 +7296,16 @@
         <v>525</v>
       </c>
       <c r="E29" t="s">
+        <v>679</v>
+      </c>
+      <c r="F29" t="s">
         <v>680</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>681</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>682</v>
-      </c>
-      <c r="H29" t="s">
-        <v>683</v>
       </c>
       <c r="I29" t="s">
         <v>15</v>
@@ -7336,16 +7331,16 @@
         <v>106</v>
       </c>
       <c r="G30" t="s">
+        <v>683</v>
+      </c>
+      <c r="H30" t="s">
         <v>684</v>
-      </c>
-      <c r="H30" t="s">
-        <v>685</v>
       </c>
       <c r="I30" t="s">
         <v>72</v>
       </c>
       <c r="J30" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -7362,13 +7357,13 @@
         <v>525</v>
       </c>
       <c r="E31" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="F31" t="s">
         <v>102</v>
       </c>
       <c r="G31" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="H31" t="s">
         <v>104</v>
@@ -7377,7 +7372,7 @@
         <v>72</v>
       </c>
       <c r="J31" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -7400,7 +7395,7 @@
         <v>123</v>
       </c>
       <c r="G32" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="H32" t="s">
         <v>125</v>
@@ -7409,7 +7404,7 @@
         <v>9</v>
       </c>
       <c r="J32" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -7432,7 +7427,7 @@
         <v>127</v>
       </c>
       <c r="G33" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="H33" t="s">
         <v>129</v>
@@ -7441,7 +7436,7 @@
         <v>72</v>
       </c>
       <c r="J33" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -7464,16 +7459,16 @@
         <v>119</v>
       </c>
       <c r="G34" t="s">
+        <v>690</v>
+      </c>
+      <c r="H34" t="s">
         <v>691</v>
-      </c>
-      <c r="H34" t="s">
-        <v>692</v>
       </c>
       <c r="I34" t="s">
         <v>72</v>
       </c>
       <c r="J34" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -7505,7 +7500,7 @@
         <v>9</v>
       </c>
       <c r="J35" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -7522,7 +7517,7 @@
         <v>525</v>
       </c>
       <c r="E36" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F36" t="s">
         <v>111</v>
@@ -7537,7 +7532,7 @@
         <v>9</v>
       </c>
       <c r="J36" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -7560,7 +7555,7 @@
         <v>131</v>
       </c>
       <c r="G37" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="H37" t="s">
         <v>133</v>
@@ -7569,7 +7564,7 @@
         <v>72</v>
       </c>
       <c r="J37" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -8313,7 +8308,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="E1:J1" xr:uid="{DE965883-0425-4F05-8072-E0B97A65FD07}"/>
+  <autoFilter ref="E1:J62" xr:uid="{DE965883-0425-4F05-8072-E0B97A65FD07}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8338,25 +8333,25 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>695</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>696</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>697</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>698</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>1</v>
@@ -8391,7 +8386,7 @@
         <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -8426,7 +8421,7 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
@@ -8461,7 +8456,7 @@
         <v>18</v>
       </c>
       <c r="G4" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H4" t="s">
         <v>19</v>
@@ -8496,7 +8491,7 @@
         <v>238</v>
       </c>
       <c r="G5" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H5" t="s">
         <v>239</v>
@@ -8531,7 +8526,7 @@
         <v>244</v>
       </c>
       <c r="G6" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H6" t="s">
         <v>245</v>
@@ -8566,7 +8561,7 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H7" t="s">
         <v>25</v>
@@ -8598,7 +8593,7 @@
         <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H8" t="s">
         <v>29</v>
@@ -8630,7 +8625,7 @@
         <v>32</v>
       </c>
       <c r="G9" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H9" t="s">
         <v>33</v>
@@ -8700,7 +8695,7 @@
         <v>43</v>
       </c>
       <c r="G11" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H11" t="s">
         <v>44</v>
@@ -8735,7 +8730,7 @@
         <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H12" t="s">
         <v>50</v>
@@ -8770,7 +8765,7 @@
         <v>53</v>
       </c>
       <c r="G13" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="H13" t="s">
         <v>54</v>
@@ -8805,7 +8800,7 @@
         <v>58</v>
       </c>
       <c r="G14" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="H14" t="s">
         <v>59</v>
@@ -8840,7 +8835,7 @@
         <v>63</v>
       </c>
       <c r="G15" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="H15" t="s">
         <v>64</v>
@@ -8875,7 +8870,7 @@
         <v>228</v>
       </c>
       <c r="G16" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H16" t="s">
         <v>29</v>
@@ -8910,7 +8905,7 @@
         <v>69</v>
       </c>
       <c r="G17" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="H17" t="s">
         <v>70</v>
@@ -8945,7 +8940,7 @@
         <v>75</v>
       </c>
       <c r="G18" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="H18" t="s">
         <v>76</v>
@@ -8980,7 +8975,7 @@
         <v>81</v>
       </c>
       <c r="G19" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="H19" t="s">
         <v>82</v>
@@ -9015,7 +9010,7 @@
         <v>230</v>
       </c>
       <c r="G20" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="H20" t="s">
         <v>88</v>
@@ -9047,7 +9042,7 @@
         <v>87</v>
       </c>
       <c r="G21" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="H21" t="s">
         <v>88</v>
@@ -9079,7 +9074,7 @@
         <v>92</v>
       </c>
       <c r="G22" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="H22" t="s">
         <v>93</v>
@@ -9114,7 +9109,7 @@
         <v>97</v>
       </c>
       <c r="G23" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="H23" t="s">
         <v>98</v>
@@ -9149,7 +9144,7 @@
         <v>102</v>
       </c>
       <c r="G24" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="H24" t="s">
         <v>103</v>
@@ -9181,7 +9176,7 @@
         <v>106</v>
       </c>
       <c r="G25" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="H25" t="s">
         <v>107</v>
@@ -9216,7 +9211,7 @@
         <v>111</v>
       </c>
       <c r="G26" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="H26" t="s">
         <v>112</v>
@@ -9251,7 +9246,7 @@
         <v>115</v>
       </c>
       <c r="G27" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="H27" t="s">
         <v>116</v>
@@ -9321,7 +9316,7 @@
         <v>123</v>
       </c>
       <c r="G29" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H29" t="s">
         <v>124</v>
@@ -9391,7 +9386,7 @@
         <v>131</v>
       </c>
       <c r="G31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="H31" t="s">
         <v>132</v>
@@ -9426,7 +9421,7 @@
         <v>136</v>
       </c>
       <c r="G32" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="H32" t="s">
         <v>137</v>
@@ -9461,7 +9456,7 @@
         <v>140</v>
       </c>
       <c r="G33" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="H33" t="s">
         <v>141</v>
@@ -9493,7 +9488,7 @@
         <v>143</v>
       </c>
       <c r="G34" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H34" t="s">
         <v>144</v>
@@ -9525,7 +9520,7 @@
         <v>232</v>
       </c>
       <c r="G35" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H35" t="s">
         <v>144</v>
@@ -9557,7 +9552,7 @@
         <v>147</v>
       </c>
       <c r="G36" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H36" t="s">
         <v>144</v>
@@ -9592,7 +9587,7 @@
         <v>150</v>
       </c>
       <c r="G37" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H37" t="s">
         <v>144</v>
@@ -9624,7 +9619,7 @@
         <v>152</v>
       </c>
       <c r="G38" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H38" t="s">
         <v>144</v>
@@ -9656,7 +9651,7 @@
         <v>154</v>
       </c>
       <c r="G39" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="H39" t="s">
         <v>155</v>
@@ -9688,7 +9683,7 @@
         <v>157</v>
       </c>
       <c r="G40" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H40" t="s">
         <v>158</v>
@@ -9720,7 +9715,7 @@
         <v>233</v>
       </c>
       <c r="G41" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H41" t="s">
         <v>158</v>
@@ -9752,7 +9747,7 @@
         <v>160</v>
       </c>
       <c r="G42" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H42" t="s">
         <v>158</v>
@@ -9784,7 +9779,7 @@
         <v>161</v>
       </c>
       <c r="G43" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H43" t="s">
         <v>158</v>
@@ -9816,7 +9811,7 @@
         <v>162</v>
       </c>
       <c r="G44" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H44" t="s">
         <v>158</v>
@@ -9848,7 +9843,7 @@
         <v>163</v>
       </c>
       <c r="G45" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="H45" t="s">
         <v>158</v>
@@ -9880,7 +9875,7 @@
         <v>165</v>
       </c>
       <c r="G46" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H46" t="s">
         <v>166</v>
@@ -9915,7 +9910,7 @@
         <v>171</v>
       </c>
       <c r="G47" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="H47" t="s">
         <v>172</v>
@@ -9950,7 +9945,7 @@
         <v>176</v>
       </c>
       <c r="G48" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H48" t="s">
         <v>177</v>
@@ -9982,7 +9977,7 @@
         <v>180</v>
       </c>
       <c r="G49" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="H49" t="s">
         <v>181</v>
@@ -10014,7 +10009,7 @@
         <v>184</v>
       </c>
       <c r="G50" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="H50" t="s">
         <v>185</v>
@@ -10046,7 +10041,7 @@
         <v>188</v>
       </c>
       <c r="G51" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="H51" t="s">
         <v>189</v>
@@ -10078,7 +10073,7 @@
         <v>192</v>
       </c>
       <c r="G52" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="H52" t="s">
         <v>193</v>
@@ -10110,7 +10105,7 @@
         <v>196</v>
       </c>
       <c r="G53" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="H53" t="s">
         <v>197</v>
@@ -10142,7 +10137,7 @@
         <v>199</v>
       </c>
       <c r="G54" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H54" t="s">
         <v>200</v>
@@ -10174,7 +10169,7 @@
         <v>203</v>
       </c>
       <c r="G55" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H55" t="s">
         <v>204</v>
@@ -10206,7 +10201,7 @@
         <v>206</v>
       </c>
       <c r="G56" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="H56" t="s">
         <v>207</v>
@@ -10238,7 +10233,7 @@
         <v>208</v>
       </c>
       <c r="G57" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H57" t="s">
         <v>209</v>
@@ -10270,7 +10265,7 @@
         <v>211</v>
       </c>
       <c r="G58" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H58" t="s">
         <v>209</v>
@@ -10302,7 +10297,7 @@
         <v>234</v>
       </c>
       <c r="G59" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H59" t="s">
         <v>209</v>
@@ -10334,7 +10329,7 @@
         <v>212</v>
       </c>
       <c r="G60" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H60" t="s">
         <v>209</v>
@@ -10366,7 +10361,7 @@
         <v>213</v>
       </c>
       <c r="G61" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H61" t="s">
         <v>209</v>
@@ -10398,7 +10393,7 @@
         <v>214</v>
       </c>
       <c r="G62" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H62" t="s">
         <v>209</v>
@@ -10430,7 +10425,7 @@
         <v>215</v>
       </c>
       <c r="G63" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H63" t="s">
         <v>209</v>
@@ -10462,7 +10457,7 @@
         <v>236</v>
       </c>
       <c r="G64" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="H64" t="s">
         <v>209</v>
@@ -10494,7 +10489,7 @@
         <v>217</v>
       </c>
       <c r="G65" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="H65" t="s">
         <v>218</v>
@@ -10529,7 +10524,7 @@
         <v>221</v>
       </c>
       <c r="G66" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="H66" t="s">
         <v>222</v>
@@ -10564,7 +10559,7 @@
         <v>224</v>
       </c>
       <c r="G67" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="H67" t="s">
         <v>225</v>

</xml_diff>